<commit_message>
housekeep-db: excel format bug fixed
</commit_message>
<xml_diff>
--- a/ecuacion-tool-housekeep-db/excel-format/housekeep-db_fmt-v2.0.0-en_sample.xlsx
+++ b/ecuacion-tool-housekeep-db/excel-format/housekeep-db_fmt-v2.0.0-en_sample.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10817"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10821"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/yosuke.tanaka/Desktop/development/git/ecuacion-tools/ecuacion-tool-housekeep-db/excel-format/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C4D10B3-A4DE-C348-8C3F-9F2D33DD8B56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC402427-3A73-9142-B457-C5035579DDE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6580" yWindow="500" windowWidth="28800" windowHeight="16640" xr2:uid="{8AED4C0F-E98F-E547-A0B0-59373B747A30}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16600" activeTab="3" xr2:uid="{8AED4C0F-E98F-E547-A0B0-59373B747A30}"/>
   </bookViews>
   <sheets>
     <sheet name="change log" sheetId="8" r:id="rId1"/>
@@ -532,20 +532,20 @@
     <xf numFmtId="14" fontId="5" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="3" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="5" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="3" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -564,6 +564,195 @@
         <sz val="11"/>
         <color theme="1"/>
         <name val="游ゴシック"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="游ゴシック"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="游ゴシック"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="游ゴシック"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="游ゴシック"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="游ゴシック"/>
+        <family val="3"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="游ゴシック"/>
+        <family val="3"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="游ゴシック"/>
+        <family val="3"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="游ゴシック"/>
+        <family val="3"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="3"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="游ゴシック"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="游ゴシック"/>
+        <family val="3"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="游ゴシック"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="游ゴシック"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="游ゴシック"/>
         <family val="3"/>
         <charset val="128"/>
         <scheme val="minor"/>
@@ -882,150 +1071,6 @@
         <strike val="0"/>
         <outline val="0"/>
         <shadow val="0"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="游ゴシック"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="游ゴシック"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="游ゴシック"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="游ゴシック"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="游ゴシック"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="游ゴシック"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="游ゴシック"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="游ゴシック"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="游ゴシック"/>
-        <family val="3"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="游ゴシック"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="游ゴシック"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
         <u val="none"/>
         <vertAlign val="baseline"/>
         <sz val="11"/>
@@ -1171,129 +1216,84 @@
         <sz val="11"/>
         <color theme="1"/>
         <name val="游ゴシック"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="游ゴシック"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="游ゴシック"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="游ゴシック"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="游ゴシック"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="游ゴシック"/>
-        <family val="3"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="游ゴシック"/>
-        <family val="3"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="游ゴシック"/>
-        <family val="3"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="游ゴシック"/>
-        <family val="3"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="3"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="游ゴシック"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="游ゴシック"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="游ゴシック"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="游ゴシック"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="游ゴシック"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="游ゴシック"/>
         <charset val="128"/>
         <scheme val="minor"/>
       </font>
@@ -1488,104 +1488,104 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{22FC8765-21CB-4449-8794-6F7BB0DF5CF4}" name="テーブル5" displayName="テーブル5" ref="A3:D5" totalsRowShown="0" headerRowDxfId="42" dataDxfId="41">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{22FC8765-21CB-4449-8794-6F7BB0DF5CF4}" name="テーブル5" displayName="テーブル5" ref="A3:D5" totalsRowShown="0" headerRowDxfId="45" dataDxfId="44">
   <autoFilter ref="A3:D5" xr:uid="{00000000-0009-0000-0100-000005000000}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{E4142994-3892-C340-9A65-88F80365D8CE}" name="Date" dataDxfId="40"/>
-    <tableColumn id="2" xr3:uid="{35BACA5E-E809-0844-BAB8-78CB7B6B343E}" name="Version" dataDxfId="39"/>
-    <tableColumn id="3" xr3:uid="{C4E826C9-5641-E048-9706-B0754516BA47}" name="Notes" dataDxfId="38"/>
-    <tableColumn id="4" xr3:uid="{10D446C7-4721-E74C-863B-894EBEBABA4B}" name="Updated By" dataDxfId="37"/>
+    <tableColumn id="1" xr3:uid="{E4142994-3892-C340-9A65-88F80365D8CE}" name="Date" dataDxfId="43"/>
+    <tableColumn id="2" xr3:uid="{35BACA5E-E809-0844-BAB8-78CB7B6B343E}" name="Version" dataDxfId="42"/>
+    <tableColumn id="3" xr3:uid="{C4E826C9-5641-E048-9706-B0754516BA47}" name="Notes" dataDxfId="41"/>
+    <tableColumn id="4" xr3:uid="{10D446C7-4721-E74C-863B-894EBEBABA4B}" name="Updated By" dataDxfId="40"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{24155060-B8ED-8845-8CC4-DA9C5F0847AB}" name="テーブル4" displayName="テーブル4" ref="A1:B3" totalsRowShown="0" headerRowDxfId="36" dataDxfId="35">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{24155060-B8ED-8845-8CC4-DA9C5F0847AB}" name="テーブル4" displayName="テーブル4" ref="A1:B3" totalsRowShown="0" headerRowDxfId="39" dataDxfId="38">
   <autoFilter ref="A1:B3" xr:uid="{24155060-B8ED-8845-8CC4-DA9C5F0847AB}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{98E4E7E5-8F2D-A64D-A202-DFFC12164331}" name="item" dataDxfId="34"/>
-    <tableColumn id="2" xr3:uid="{E3BF9435-59E2-8948-93E9-5462EEBA2F6D}" name="value" dataDxfId="33"/>
+    <tableColumn id="1" xr3:uid="{98E4E7E5-8F2D-A64D-A202-DFFC12164331}" name="item" dataDxfId="37"/>
+    <tableColumn id="2" xr3:uid="{E3BF9435-59E2-8948-93E9-5462EEBA2F6D}" name="value" dataDxfId="36"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{DD7B5D78-5E9B-DE4B-B691-1DF452AB1374}" name="テーブル3" displayName="テーブル3" ref="A5:I6" insertRow="1" totalsRowShown="0" headerRowDxfId="32" dataDxfId="31">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{DD7B5D78-5E9B-DE4B-B691-1DF452AB1374}" name="テーブル3" displayName="テーブル3" ref="A5:I6" insertRow="1" totalsRowShown="0" headerRowDxfId="56" dataDxfId="55">
   <autoFilter ref="A5:I6" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{6F9607F2-5B3B-AC43-9B81-3332FF1A0DAD}" name="DB Connection ID" dataDxfId="30" dataCellStyle="標準 2"/>
-    <tableColumn id="2" xr3:uid="{EB1F7206-30E2-EA43-A8CF-9AD4F9A14E33}" name="Driver Name" dataDxfId="29"/>
-    <tableColumn id="3" xr3:uid="{4D55D82B-BDD3-2B46-A21D-0450B9F1910B}" name="Connection URL: Protocol" dataDxfId="28" dataCellStyle="標準 2"/>
-    <tableColumn id="4" xr3:uid="{84D0845B-C5EE-9047-A1AB-EE336A75EBAD}" name="Connection URL: Server" dataDxfId="27" dataCellStyle="標準 2"/>
-    <tableColumn id="5" xr3:uid="{6197D9F5-186B-D44E-ADCB-89378D8B3702}" name="Connection URL: Port" dataDxfId="26" dataCellStyle="標準 2"/>
-    <tableColumn id="6" xr3:uid="{26B865D4-D13A-9C4C-B104-C634122F988F}" name="Connection URL: Database" dataDxfId="25" dataCellStyle="標準 2"/>
-    <tableColumn id="7" xr3:uid="{046864C3-26A2-7B44-B07A-EAB68FAF2EEA}" name="Connection URL: Schema" dataDxfId="24" dataCellStyle="標準 2"/>
-    <tableColumn id="8" xr3:uid="{4A5FE8C4-A0F3-3E4A-9BB5-642C226504CF}" name="Username" dataDxfId="23" dataCellStyle="標準 2"/>
-    <tableColumn id="9" xr3:uid="{6A963E93-AA2B-944F-A127-0CD6F7E61369}" name="Password" dataDxfId="22" dataCellStyle="標準 2"/>
+    <tableColumn id="1" xr3:uid="{6F9607F2-5B3B-AC43-9B81-3332FF1A0DAD}" name="DB Connection ID" dataDxfId="54" dataCellStyle="標準 2"/>
+    <tableColumn id="2" xr3:uid="{EB1F7206-30E2-EA43-A8CF-9AD4F9A14E33}" name="Driver Name" dataDxfId="53"/>
+    <tableColumn id="3" xr3:uid="{4D55D82B-BDD3-2B46-A21D-0450B9F1910B}" name="Connection URL: Protocol" dataDxfId="52" dataCellStyle="標準 2"/>
+    <tableColumn id="4" xr3:uid="{84D0845B-C5EE-9047-A1AB-EE336A75EBAD}" name="Connection URL: Server" dataDxfId="51" dataCellStyle="標準 2"/>
+    <tableColumn id="5" xr3:uid="{6197D9F5-186B-D44E-ADCB-89378D8B3702}" name="Connection URL: Port" dataDxfId="50" dataCellStyle="標準 2"/>
+    <tableColumn id="6" xr3:uid="{26B865D4-D13A-9C4C-B104-C634122F988F}" name="Connection URL: Database" dataDxfId="49" dataCellStyle="標準 2"/>
+    <tableColumn id="7" xr3:uid="{046864C3-26A2-7B44-B07A-EAB68FAF2EEA}" name="Connection URL: Schema" dataDxfId="48" dataCellStyle="標準 2"/>
+    <tableColumn id="8" xr3:uid="{4A5FE8C4-A0F3-3E4A-9BB5-642C226504CF}" name="Username" dataDxfId="47" dataCellStyle="標準 2"/>
+    <tableColumn id="9" xr3:uid="{6A963E93-AA2B-944F-A127-0CD6F7E61369}" name="Password" dataDxfId="46" dataCellStyle="標準 2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{61C29F33-44CC-B14C-8562-09C29609B4D7}" name="テーブル32" displayName="テーブル32" ref="A5:O6" totalsRowShown="0" headerRowDxfId="21" dataDxfId="20">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{61C29F33-44CC-B14C-8562-09C29609B4D7}" name="テーブル32" displayName="テーブル32" ref="A5:O6" totalsRowShown="0" headerRowDxfId="35" dataDxfId="34">
   <autoFilter ref="A5:O6" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
   <tableColumns count="15">
-    <tableColumn id="1" xr3:uid="{CBD51E9F-618C-754C-8BA6-0B46FCE3F82F}" name="Task ID" dataDxfId="19"/>
-    <tableColumn id="12" xr3:uid="{5E33A481-4C3C-A049-B253-3EC944DDB6EC}" name="DB Connection ID" dataDxfId="18" dataCellStyle="標準 2"/>
-    <tableColumn id="2" xr3:uid="{AADC801E-ABC4-9E4F-8EFF-3383030B2A4B}" name="Soft / Hard Delete" dataDxfId="17"/>
-    <tableColumn id="15" xr3:uid="{C9A2944C-947B-B844-AE98-12A7D9A1D364}" name="Soft / Hard Delete (internal value)" dataDxfId="16">
+    <tableColumn id="1" xr3:uid="{CBD51E9F-618C-754C-8BA6-0B46FCE3F82F}" name="Task ID" dataDxfId="33"/>
+    <tableColumn id="12" xr3:uid="{5E33A481-4C3C-A049-B253-3EC944DDB6EC}" name="DB Connection ID" dataDxfId="32" dataCellStyle="標準 2"/>
+    <tableColumn id="2" xr3:uid="{AADC801E-ABC4-9E4F-8EFF-3383030B2A4B}" name="Soft / Hard Delete" dataDxfId="31"/>
+    <tableColumn id="15" xr3:uid="{C9A2944C-947B-B844-AE98-12A7D9A1D364}" name="Soft / Hard Delete (internal value)" dataDxfId="30">
       <calculatedColumnFormula array="1">_xlfn.IFS(テーブル32[[#This Row],[Soft / Hard Delete]]="Soft Delete","SOFT_DELETE",テーブル32[[#This Row],[Soft / Hard Delete]]="Hard Delete","HARD_DELETE",TRUE,"")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{6C98AD64-A3D3-F44E-A881-8EFCEA1F9F67}" name="Table Name" dataDxfId="15" dataCellStyle="標準 2"/>
-    <tableColumn id="4" xr3:uid="{A38A3149-447A-8548-9729-49CE9E074B36}" name="ID Column Name" dataDxfId="14" dataCellStyle="標準 2"/>
-    <tableColumn id="10" xr3:uid="{B15AF0F8-272C-B943-9D75-81A8797BC598}" name="ID Column Literal Symbol" dataDxfId="13"/>
-    <tableColumn id="5" xr3:uid="{6FE6A1FF-15C9-7545-B254-7B2C29EF168D}" name="Expiration Check: Timestamp Column Name" dataDxfId="12" dataCellStyle="標準 2"/>
-    <tableColumn id="11" xr3:uid="{BF075527-A2E7-834B-AD05-1A2D9E3BA0AD}" name="Expiration Check: Timestamp Column Data Type" dataDxfId="11"/>
-    <tableColumn id="6" xr3:uid="{94EB7746-8D75-EE47-A2F3-81D397D26AE1}" name="Expiration Check: Validity Days" dataDxfId="10" dataCellStyle="標準 2"/>
-    <tableColumn id="7" xr3:uid="{62ADB4F3-1C59-7F4B-819E-B49B0ABB889C}" name="Soft Delete Column Name" dataDxfId="9" dataCellStyle="標準 2"/>
-    <tableColumn id="8" xr3:uid="{0EB6A694-7E00-B64C-AF69-22B6C7E1C560}" name="Soft Delete: Update Timestamp Column Name" dataDxfId="8" dataCellStyle="標準 2"/>
-    <tableColumn id="9" xr3:uid="{0A6924E1-C0CB-AF40-A208-E0E96A257245}" name="Soft Delete: Update User ID Column Name" dataDxfId="7" dataCellStyle="標準 2"/>
-    <tableColumn id="14" xr3:uid="{93BF3B4F-D2E8-A640-A768-A230439878D9}" name="Soft Delete: Update User ID Column Literal Symbol" dataDxfId="6" dataCellStyle="標準 2"/>
-    <tableColumn id="13" xr3:uid="{DE6ACC44-9137-0840-9711-E0D04FCC851F}" name="Soft Delete: Update User ID Column Value" dataDxfId="5" dataCellStyle="標準 2"/>
+    <tableColumn id="3" xr3:uid="{6C98AD64-A3D3-F44E-A881-8EFCEA1F9F67}" name="Table Name" dataDxfId="29" dataCellStyle="標準 2"/>
+    <tableColumn id="4" xr3:uid="{A38A3149-447A-8548-9729-49CE9E074B36}" name="ID Column Name" dataDxfId="28" dataCellStyle="標準 2"/>
+    <tableColumn id="10" xr3:uid="{B15AF0F8-272C-B943-9D75-81A8797BC598}" name="ID Column Literal Symbol" dataDxfId="27"/>
+    <tableColumn id="5" xr3:uid="{6FE6A1FF-15C9-7545-B254-7B2C29EF168D}" name="Expiration Check: Timestamp Column Name" dataDxfId="26" dataCellStyle="標準 2"/>
+    <tableColumn id="11" xr3:uid="{BF075527-A2E7-834B-AD05-1A2D9E3BA0AD}" name="Expiration Check: Timestamp Column Data Type" dataDxfId="25"/>
+    <tableColumn id="6" xr3:uid="{94EB7746-8D75-EE47-A2F3-81D397D26AE1}" name="Expiration Check: Validity Days" dataDxfId="24" dataCellStyle="標準 2"/>
+    <tableColumn id="7" xr3:uid="{62ADB4F3-1C59-7F4B-819E-B49B0ABB889C}" name="Soft Delete Column Name" dataDxfId="23" dataCellStyle="標準 2"/>
+    <tableColumn id="8" xr3:uid="{0EB6A694-7E00-B64C-AF69-22B6C7E1C560}" name="Soft Delete: Update Timestamp Column Name" dataDxfId="22" dataCellStyle="標準 2"/>
+    <tableColumn id="9" xr3:uid="{0A6924E1-C0CB-AF40-A208-E0E96A257245}" name="Soft Delete: Update User ID Column Name" dataDxfId="21" dataCellStyle="標準 2"/>
+    <tableColumn id="14" xr3:uid="{93BF3B4F-D2E8-A640-A768-A230439878D9}" name="Soft Delete: Update User ID Column Literal Symbol" dataDxfId="20" dataCellStyle="標準 2"/>
+    <tableColumn id="13" xr3:uid="{DE6ACC44-9137-0840-9711-E0D04FCC851F}" name="Soft Delete: Update User ID Column Value" dataDxfId="19" dataCellStyle="標準 2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{DBD8E589-22D9-8541-A9D6-F03C8FC47C4E}" name="テーブル323" displayName="テーブル323" ref="A5:D6" insertRow="1" totalsRowShown="0" headerRowDxfId="4">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{DBD8E589-22D9-8541-A9D6-F03C8FC47C4E}" name="テーブル323" displayName="テーブル323" ref="A5:D6" insertRow="1" totalsRowShown="0" headerRowDxfId="18">
   <autoFilter ref="A5:D6" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{0B02141A-0F5F-8849-982C-6C0A6A7BEE4F}" name="Task ID" dataDxfId="3" dataCellStyle="標準 2"/>
-    <tableColumn id="12" xr3:uid="{69A08ECC-4076-9E48-8CE9-3FABB073CA81}" name="Search Condition Column Name" dataDxfId="2"/>
-    <tableColumn id="2" xr3:uid="{511F37DB-74E3-394C-9204-B1C6CA623CD0}" name="Search Condtion Column Literal Symbol" dataDxfId="1"/>
-    <tableColumn id="3" xr3:uid="{2F474AF9-6428-D446-9D8C-0FEF2C86FE1D}" name="Search Condition Column Value" dataDxfId="0" dataCellStyle="標準 2"/>
+    <tableColumn id="1" xr3:uid="{0B02141A-0F5F-8849-982C-6C0A6A7BEE4F}" name="Task ID" dataDxfId="17" dataCellStyle="標準 2"/>
+    <tableColumn id="12" xr3:uid="{69A08ECC-4076-9E48-8CE9-3FABB073CA81}" name="Search Condition Column Name" dataDxfId="16"/>
+    <tableColumn id="2" xr3:uid="{511F37DB-74E3-394C-9204-B1C6CA623CD0}" name="Search Condtion Column Literal Symbol" dataDxfId="15"/>
+    <tableColumn id="3" xr3:uid="{2F474AF9-6428-D446-9D8C-0FEF2C86FE1D}" name="Search Condition Column Value" dataDxfId="14" dataCellStyle="標準 2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{5EE7E132-481E-3140-932F-4C153EC6948B}" name="テーブル3236" displayName="テーブル3236" ref="A5:L6" totalsRowShown="0" headerRowDxfId="56" dataDxfId="55">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{5EE7E132-481E-3140-932F-4C153EC6948B}" name="テーブル3236" displayName="テーブル3236" ref="A5:L6" totalsRowShown="0" headerRowDxfId="13" dataDxfId="12">
   <autoFilter ref="A5:L6" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
   <tableColumns count="12">
-    <tableColumn id="1" xr3:uid="{65C86A53-0A13-8F47-916D-E06475BCECE3}" name="Task ID" dataDxfId="54"/>
-    <tableColumn id="12" xr3:uid="{987F2B9C-94EA-9F41-A4C1-6D7606B12BAC}" name="Related Table Process Pattern" dataDxfId="53"/>
-    <tableColumn id="10" xr3:uid="{B871A9E9-220D-F74C-A1C5-BED1ED6DD954}" name="Related Table Process Pattern (internal value)" dataDxfId="52">
+    <tableColumn id="1" xr3:uid="{65C86A53-0A13-8F47-916D-E06475BCECE3}" name="Task ID" dataDxfId="11"/>
+    <tableColumn id="12" xr3:uid="{987F2B9C-94EA-9F41-A4C1-6D7606B12BAC}" name="Related Table Process Pattern" dataDxfId="10"/>
+    <tableColumn id="10" xr3:uid="{B871A9E9-220D-F74C-A1C5-BED1ED6DD954}" name="Related Table Process Pattern (internal value)" dataDxfId="9">
       <calculatedColumnFormula array="1">_xlfn.IFS(テーブル3236[[#This Row],[Related Table Process Pattern]]="Delete","DELETE",テーブル3236[[#This Row],[Related Table Process Pattern]]="Check and Skip Delete","CHECK_AND_SKIP_DELETE",TRUE,"")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="13" xr3:uid="{5E73C8D1-B2FA-854B-BEBB-60B6E93A2638}" name="Target Table Column Name" dataDxfId="51"/>
-    <tableColumn id="2" xr3:uid="{3B40126A-13DD-E04B-A86B-9387EB6006A1}" name="Related Table Name" dataDxfId="50" dataCellStyle="標準 2"/>
-    <tableColumn id="3" xr3:uid="{59ED585B-1BCF-DB41-A333-2655E74C710D}" name="Related Table ID Column Name" dataDxfId="49" dataCellStyle="標準 2"/>
-    <tableColumn id="14" xr3:uid="{75144EA6-AFC2-3646-9A0E-DD4A2D917411}" name="Related Table ID Column Literal Symbol" dataDxfId="48" dataCellStyle="標準 2"/>
-    <tableColumn id="4" xr3:uid="{684AF203-54CE-5A42-8441-2636BF604DAF}" name="Soft Delete Column Name" dataDxfId="47" dataCellStyle="標準 2"/>
-    <tableColumn id="5" xr3:uid="{1D070257-74D6-6746-B460-ACB59A1770E6}" name="Soft Delete: Update Timestamp Column Name" dataDxfId="46" dataCellStyle="標準 2"/>
-    <tableColumn id="6" xr3:uid="{59287FEB-061F-B946-B814-312CDD2F482D}" name="Soft Delete: Update User ID Column Name" dataDxfId="45" dataCellStyle="標準 2"/>
-    <tableColumn id="7" xr3:uid="{E0734288-8DC3-C342-98A6-DBC50A55CEF9}" name="Soft Delete: Update User ID Column Literal Symbol" dataDxfId="44" dataCellStyle="標準 2"/>
-    <tableColumn id="8" xr3:uid="{D5E8A958-B06D-554D-B183-49DD307AC86A}" name="Soft Delete: Update User ID Column Value" dataDxfId="43" dataCellStyle="標準 2"/>
+    <tableColumn id="13" xr3:uid="{5E73C8D1-B2FA-854B-BEBB-60B6E93A2638}" name="Target Table Column Name" dataDxfId="8"/>
+    <tableColumn id="2" xr3:uid="{3B40126A-13DD-E04B-A86B-9387EB6006A1}" name="Related Table Name" dataDxfId="7" dataCellStyle="標準 2"/>
+    <tableColumn id="3" xr3:uid="{59ED585B-1BCF-DB41-A333-2655E74C710D}" name="Related Table ID Column Name" dataDxfId="6" dataCellStyle="標準 2"/>
+    <tableColumn id="14" xr3:uid="{75144EA6-AFC2-3646-9A0E-DD4A2D917411}" name="Related Table ID Column Literal Symbol" dataDxfId="5" dataCellStyle="標準 2"/>
+    <tableColumn id="4" xr3:uid="{684AF203-54CE-5A42-8441-2636BF604DAF}" name="Soft Delete Column Name" dataDxfId="4" dataCellStyle="標準 2"/>
+    <tableColumn id="5" xr3:uid="{1D070257-74D6-6746-B460-ACB59A1770E6}" name="Soft Delete: Update Timestamp Column Name" dataDxfId="3" dataCellStyle="標準 2"/>
+    <tableColumn id="6" xr3:uid="{59287FEB-061F-B946-B814-312CDD2F482D}" name="Soft Delete: Update User ID Column Name" dataDxfId="2" dataCellStyle="標準 2"/>
+    <tableColumn id="7" xr3:uid="{E0734288-8DC3-C342-98A6-DBC50A55CEF9}" name="Soft Delete: Update User ID Column Literal Symbol" dataDxfId="1" dataCellStyle="標準 2"/>
+    <tableColumn id="8" xr3:uid="{D5E8A958-B06D-554D-B183-49DD307AC86A}" name="Soft Delete: Update User ID Column Value" dataDxfId="0" dataCellStyle="標準 2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1938,7 +1938,7 @@
       <c r="B5" s="22" t="s">
         <v>70</v>
       </c>
-      <c r="C5" s="28" t="s">
+      <c r="C5" s="24" t="s">
         <v>71</v>
       </c>
       <c r="D5" s="11" t="s">
@@ -2286,20 +2286,20 @@
       </c>
       <c r="F4" s="25"/>
       <c r="G4" s="25"/>
-      <c r="H4" s="24" t="s">
+      <c r="H4" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="I4" s="24"/>
-      <c r="J4" s="24"/>
+      <c r="I4" s="27"/>
+      <c r="J4" s="27"/>
       <c r="K4" s="19" t="s">
         <v>7</v>
       </c>
-      <c r="L4" s="27" t="s">
+      <c r="L4" s="28" t="s">
         <v>8</v>
       </c>
-      <c r="M4" s="27"/>
-      <c r="N4" s="27"/>
-      <c r="O4" s="27"/>
+      <c r="M4" s="28"/>
+      <c r="N4" s="28"/>
+      <c r="O4" s="28"/>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A5" s="6" t="s">
@@ -2567,13 +2567,13 @@
       <c r="E4" s="25"/>
       <c r="F4" s="25"/>
       <c r="G4" s="25"/>
-      <c r="H4" s="24" t="s">
+      <c r="H4" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="I4" s="24"/>
-      <c r="J4" s="24"/>
-      <c r="K4" s="24"/>
-      <c r="L4" s="24"/>
+      <c r="I4" s="27"/>
+      <c r="J4" s="27"/>
+      <c r="K4" s="27"/>
+      <c r="L4" s="27"/>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A5" s="6" t="s">

</xml_diff>